<commit_message>
bedarfsdeckung ohne speicher 1.0
</commit_message>
<xml_diff>
--- a/data/Vergleichstabelle.xlsx
+++ b/data/Vergleichstabelle.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HansisRasanterRaser\Desktop\UNI\000_DA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HansisRasanterRaser\Desktop\UNI\000_DA\git\knEBiD\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{570390D4-D34A-46B2-80A9-876039DD8CAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0039BA81-A374-47EA-AFA7-CF15BFADE579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{795E655B-2E8D-4399-964B-0D83E41554F5}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{795E655B-2E8D-4399-964B-0D83E41554F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Stom" sheetId="1" r:id="rId1"/>
@@ -1246,7 +1246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1259,9 +1259,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="6" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1807,7 +1805,7 @@
       <c r="N9" s="5">
         <v>46</v>
       </c>
-      <c r="O9" s="13">
+      <c r="O9" s="12">
         <v>6250</v>
       </c>
       <c r="P9" s="5">
@@ -1846,7 +1844,7 @@
       <c r="K11" t="s">
         <v>33</v>
       </c>
-      <c r="M11" s="12">
+      <c r="M11" s="5">
         <v>1</v>
       </c>
     </row>
@@ -2114,10 +2112,9 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="9"/>
-      <c r="C6" s="14" t="s">
+      <c r="C6" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="14"/>
       <c r="E6" t="s">
         <v>76</v>
       </c>

</xml_diff>